<commit_message>
Testes e correções de erros. Criação de documentos para a apresentação
</commit_message>
<xml_diff>
--- a/docs/Levantamentos de requisitos em Excel.xlsx
+++ b/docs/Levantamentos de requisitos em Excel.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30126"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30210"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/1d8aee91a57a6f63/_Pessoal/_Dar Formação/IEFP/Amadora/6 - UFCD - 10790 - Projeto de programação/1 - Conteudos/Aula 1/Tarefas/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="111" documentId="13_ncr:1_{78219426-E1C7-4A4B-B939-2F6F9581879F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{52F5BEFF-2CC8-4247-91A5-C17E16AAFBD7}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{550C6F33-077A-419C-A5D0-26D0408E17B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" firstSheet="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Req. Funcionais (RF)" sheetId="1" r:id="rId1"/>
@@ -80,7 +80,7 @@
     <t>Alta</t>
   </si>
   <si>
-    <t>Pendente</t>
+    <t>Concluido</t>
   </si>
   <si>
     <t>RF02</t>
@@ -643,6 +643,24 @@
     <xf numFmtId="0" fontId="20" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -652,29 +670,11 @@
     <xf numFmtId="0" fontId="3" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="16" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -954,22 +954,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="25.5" customHeight="1">
-      <c r="A1" s="30" t="s">
+      <c r="A1" s="28" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="30"/>
-      <c r="C1" s="30"/>
-      <c r="D1" s="30"/>
-      <c r="E1" s="30"/>
+      <c r="B1" s="28"/>
+      <c r="C1" s="28"/>
+      <c r="D1" s="28"/>
+      <c r="E1" s="28"/>
     </row>
     <row r="2" spans="1:5" ht="18" customHeight="1">
-      <c r="A2" s="31" t="s">
+      <c r="A2" s="29" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="31"/>
-      <c r="C2" s="31"/>
-      <c r="D2" s="31"/>
-      <c r="E2" s="31"/>
+      <c r="B2" s="29"/>
+      <c r="C2" s="29"/>
+      <c r="D2" s="29"/>
+      <c r="E2" s="29"/>
     </row>
     <row r="3" spans="1:5" ht="6" customHeight="1"/>
     <row r="4" spans="1:5" ht="21.75" customHeight="1">
@@ -993,10 +993,10 @@
       <c r="A5" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B5" s="35" t="s">
+      <c r="B5" s="27" t="s">
         <v>8</v>
       </c>
-      <c r="C5" s="35" t="s">
+      <c r="C5" s="27" t="s">
         <v>9</v>
       </c>
       <c r="D5" s="3" t="s">
@@ -1010,10 +1010,10 @@
       <c r="A6" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="B6" s="35" t="s">
+      <c r="B6" s="27" t="s">
         <v>13</v>
       </c>
-      <c r="C6" s="35" t="s">
+      <c r="C6" s="27" t="s">
         <v>14</v>
       </c>
       <c r="D6" s="3" t="s">
@@ -1027,10 +1027,10 @@
       <c r="A7" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B7" s="35" t="s">
+      <c r="B7" s="27" t="s">
         <v>16</v>
       </c>
-      <c r="C7" s="35" t="s">
+      <c r="C7" s="27" t="s">
         <v>17</v>
       </c>
       <c r="D7" s="6" t="s">
@@ -1044,10 +1044,10 @@
       <c r="A8" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="B8" s="34" t="s">
+      <c r="B8" s="26" t="s">
         <v>20</v>
       </c>
-      <c r="C8" s="34" t="s">
+      <c r="C8" s="26" t="s">
         <v>21</v>
       </c>
       <c r="D8" s="3" t="s">
@@ -1061,10 +1061,10 @@
       <c r="A9" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="B9" s="34" t="s">
+      <c r="B9" s="26" t="s">
         <v>23</v>
       </c>
-      <c r="C9" s="34" t="s">
+      <c r="C9" s="26" t="s">
         <v>24</v>
       </c>
       <c r="D9" s="6" t="s">
@@ -1078,10 +1078,10 @@
       <c r="A10" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="B10" s="34" t="s">
+      <c r="B10" s="26" t="s">
         <v>26</v>
       </c>
-      <c r="C10" s="34" t="s">
+      <c r="C10" s="26" t="s">
         <v>27</v>
       </c>
       <c r="D10" s="3" t="s">
@@ -1095,10 +1095,10 @@
       <c r="A11" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="B11" s="34" t="s">
+      <c r="B11" s="26" t="s">
         <v>29</v>
       </c>
-      <c r="C11" s="34" t="s">
+      <c r="C11" s="26" t="s">
         <v>30</v>
       </c>
       <c r="D11" s="3" t="s">
@@ -1112,10 +1112,10 @@
       <c r="A12" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="B12" s="34" t="s">
+      <c r="B12" s="26" t="s">
         <v>32</v>
       </c>
-      <c r="C12" s="34" t="s">
+      <c r="C12" s="26" t="s">
         <v>33</v>
       </c>
       <c r="D12" s="6" t="s">
@@ -1129,10 +1129,10 @@
       <c r="A13" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="B13" s="34" t="s">
+      <c r="B13" s="26" t="s">
         <v>35</v>
       </c>
-      <c r="C13" s="34" t="s">
+      <c r="C13" s="26" t="s">
         <v>36</v>
       </c>
       <c r="D13" s="14" t="s">
@@ -1143,25 +1143,25 @@
       </c>
     </row>
     <row r="14" spans="1:5" ht="19.5" customHeight="1">
-      <c r="A14" s="36" t="s">
+      <c r="A14" s="30" t="s">
         <v>38</v>
       </c>
-      <c r="B14" s="36"/>
-      <c r="C14" s="36"/>
-      <c r="D14" s="36"/>
+      <c r="B14" s="30"/>
+      <c r="C14" s="30"/>
+      <c r="D14" s="30"/>
       <c r="E14" s="10">
         <f>COUNTA(A5:A13)</f>
         <v>9</v>
       </c>
     </row>
     <row r="15" spans="1:5">
-      <c r="A15" s="29" t="s">
+      <c r="A15" s="31" t="s">
         <v>39</v>
       </c>
-      <c r="B15" s="29"/>
-      <c r="C15" s="29"/>
-      <c r="D15" s="29"/>
-      <c r="E15" s="29"/>
+      <c r="B15" s="31"/>
+      <c r="C15" s="31"/>
+      <c r="D15" s="31"/>
+      <c r="E15" s="31"/>
     </row>
     <row r="16" spans="1:5" ht="18" customHeight="1"/>
   </sheetData>
@@ -1203,24 +1203,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="25.5" customHeight="1">
-      <c r="A1" s="26" t="s">
+      <c r="A1" s="32" t="s">
         <v>40</v>
       </c>
-      <c r="B1" s="26"/>
-      <c r="C1" s="26"/>
-      <c r="D1" s="26"/>
-      <c r="E1" s="26"/>
-      <c r="F1" s="26"/>
+      <c r="B1" s="32"/>
+      <c r="C1" s="32"/>
+      <c r="D1" s="32"/>
+      <c r="E1" s="32"/>
+      <c r="F1" s="32"/>
     </row>
     <row r="2" spans="1:6" ht="18" customHeight="1">
-      <c r="A2" s="27" t="s">
+      <c r="A2" s="33" t="s">
         <v>41</v>
       </c>
-      <c r="B2" s="27"/>
-      <c r="C2" s="27"/>
-      <c r="D2" s="27"/>
-      <c r="E2" s="27"/>
-      <c r="F2" s="27"/>
+      <c r="B2" s="33"/>
+      <c r="C2" s="33"/>
+      <c r="D2" s="33"/>
+      <c r="E2" s="33"/>
+      <c r="F2" s="33"/>
     </row>
     <row r="3" spans="1:6" ht="6" customHeight="1"/>
     <row r="4" spans="1:6" ht="21.75" customHeight="1">
@@ -1244,10 +1244,10 @@
       <c r="A5" s="12" t="s">
         <v>43</v>
       </c>
-      <c r="B5" s="35" t="s">
+      <c r="B5" s="27" t="s">
         <v>8</v>
       </c>
-      <c r="C5" s="35" t="s">
+      <c r="C5" s="27" t="s">
         <v>9</v>
       </c>
       <c r="D5" s="3" t="s">
@@ -1261,10 +1261,10 @@
       <c r="A6" s="13" t="s">
         <v>44</v>
       </c>
-      <c r="B6" s="35" t="s">
+      <c r="B6" s="27" t="s">
         <v>13</v>
       </c>
-      <c r="C6" s="35" t="s">
+      <c r="C6" s="27" t="s">
         <v>14</v>
       </c>
       <c r="D6" s="3" t="s">
@@ -1278,10 +1278,10 @@
       <c r="A7" s="12" t="s">
         <v>45</v>
       </c>
-      <c r="B7" s="35" t="s">
+      <c r="B7" s="27" t="s">
         <v>16</v>
       </c>
-      <c r="C7" s="35" t="s">
+      <c r="C7" s="27" t="s">
         <v>17</v>
       </c>
       <c r="D7" s="6" t="s">
@@ -1295,10 +1295,10 @@
       <c r="A8" s="13" t="s">
         <v>46</v>
       </c>
-      <c r="B8" s="34" t="s">
+      <c r="B8" s="26" t="s">
         <v>20</v>
       </c>
-      <c r="C8" s="34" t="s">
+      <c r="C8" s="26" t="s">
         <v>21</v>
       </c>
       <c r="D8" s="3" t="s">
@@ -1312,10 +1312,10 @@
       <c r="A9" s="12" t="s">
         <v>47</v>
       </c>
-      <c r="B9" s="34" t="s">
+      <c r="B9" s="26" t="s">
         <v>23</v>
       </c>
-      <c r="C9" s="34" t="s">
+      <c r="C9" s="26" t="s">
         <v>24</v>
       </c>
       <c r="D9" s="6" t="s">
@@ -1329,10 +1329,10 @@
       <c r="A10" s="15" t="s">
         <v>48</v>
       </c>
-      <c r="B10" s="34" t="s">
+      <c r="B10" s="26" t="s">
         <v>26</v>
       </c>
-      <c r="C10" s="34" t="s">
+      <c r="C10" s="26" t="s">
         <v>27</v>
       </c>
       <c r="D10" s="3" t="s">
@@ -1346,10 +1346,10 @@
       <c r="A11" s="15" t="s">
         <v>49</v>
       </c>
-      <c r="B11" s="34" t="s">
+      <c r="B11" s="26" t="s">
         <v>29</v>
       </c>
-      <c r="C11" s="34" t="s">
+      <c r="C11" s="26" t="s">
         <v>30</v>
       </c>
       <c r="D11" s="3" t="s">
@@ -1364,10 +1364,10 @@
       <c r="A12" s="15" t="s">
         <v>50</v>
       </c>
-      <c r="B12" s="34" t="s">
+      <c r="B12" s="26" t="s">
         <v>32</v>
       </c>
-      <c r="C12" s="34" t="s">
+      <c r="C12" s="26" t="s">
         <v>33</v>
       </c>
       <c r="D12" s="6" t="s">
@@ -1382,10 +1382,10 @@
       <c r="A13" s="15" t="s">
         <v>51</v>
       </c>
-      <c r="B13" s="34" t="s">
+      <c r="B13" s="26" t="s">
         <v>35</v>
       </c>
-      <c r="C13" s="34" t="s">
+      <c r="C13" s="26" t="s">
         <v>36</v>
       </c>
       <c r="D13" s="14" t="s">
@@ -1397,12 +1397,12 @@
       <c r="F13" s="9"/>
     </row>
     <row r="14" spans="1:6" ht="19.5" customHeight="1">
-      <c r="A14" s="28" t="s">
+      <c r="A14" s="34" t="s">
         <v>52</v>
       </c>
-      <c r="B14" s="28"/>
-      <c r="C14" s="28"/>
-      <c r="D14" s="28"/>
+      <c r="B14" s="34"/>
+      <c r="C14" s="34"/>
+      <c r="D14" s="34"/>
       <c r="E14" s="16">
         <f>COUNTA(A5:A13)</f>
         <v>9</v>
@@ -1410,14 +1410,14 @@
       <c r="F14" s="17"/>
     </row>
     <row r="16" spans="1:6" ht="18" customHeight="1">
-      <c r="A16" s="29" t="s">
+      <c r="A16" s="31" t="s">
         <v>39</v>
       </c>
-      <c r="B16" s="29"/>
-      <c r="C16" s="29"/>
-      <c r="D16" s="29"/>
-      <c r="E16" s="29"/>
-      <c r="F16" s="29"/>
+      <c r="B16" s="31"/>
+      <c r="C16" s="31"/>
+      <c r="D16" s="31"/>
+      <c r="E16" s="31"/>
+      <c r="F16" s="31"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -1431,7 +1431,7 @@
       <formula1>"Alta,Média,Baixa"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation type="list" sqref="E5:E13" xr:uid="{00000000-0002-0000-0100-000001000000}">
+    <dataValidation type="list" sqref="E5:E13" xr:uid="{90043F91-33A7-4D5F-8394-452D229E7944}">
       <formula1>"Pendente,Em curso,Concluído,Cancelado"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -1451,22 +1451,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="30" customHeight="1">
-      <c r="A1" s="32" t="s">
+      <c r="A1" s="35" t="s">
         <v>53</v>
       </c>
-      <c r="B1" s="32"/>
-      <c r="C1" s="32"/>
-      <c r="D1" s="32"/>
-      <c r="E1" s="32"/>
+      <c r="B1" s="35"/>
+      <c r="C1" s="35"/>
+      <c r="D1" s="35"/>
+      <c r="E1" s="35"/>
     </row>
     <row r="2" spans="1:5" ht="18" customHeight="1">
-      <c r="A2" s="33" t="s">
+      <c r="A2" s="36" t="s">
         <v>54</v>
       </c>
-      <c r="B2" s="33"/>
-      <c r="C2" s="33"/>
-      <c r="D2" s="33"/>
-      <c r="E2" s="33"/>
+      <c r="B2" s="36"/>
+      <c r="C2" s="36"/>
+      <c r="D2" s="36"/>
+      <c r="E2" s="36"/>
     </row>
     <row r="3" spans="1:5" ht="9.75" customHeight="1"/>
     <row r="4" spans="1:5" ht="19.5" customHeight="1">

</xml_diff>